<commit_message>
Session 8: Fix report integrity, mechanical gates, loom tests, scale differential, TPC-H SF1, and LSM durability
</commit_message>
<xml_diff>
--- a/evidence/workbooks/04_Columnar_Query_Engine_ULTIMATE_145_Master_STATUS.xlsx
+++ b/evidence/workbooks/04_Columnar_Query_Engine_ULTIMATE_145_Master_STATUS.xlsx
@@ -20095,7 +20095,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-10-01 20:53:30</t>
+          <t>2026-10-01 21:18:35</t>
         </is>
       </c>
     </row>
@@ -20107,7 +20107,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>aa2b944</t>
+          <t>49adde6</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Session 9: Integrity repair, semantic audit, master workbook alignment, morsel parallelism, compaction and recovery
</commit_message>
<xml_diff>
--- a/evidence/workbooks/04_Columnar_Query_Engine_ULTIMATE_145_Master_STATUS.xlsx
+++ b/evidence/workbooks/04_Columnar_Query_Engine_ULTIMATE_145_Master_STATUS.xlsx
@@ -1994,31 +1994,23 @@
           <t>04-025</t>
         </is>
       </c>
-      <c r="J29" s="9" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="K29" s="9" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="J29" s="8" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="K29" s="8" t="inlineStr">
+        <is>
+          <t>✗</t>
         </is>
       </c>
       <c r="L29" s="7" t="inlineStr">
         <is>
-          <t>Verified</t>
-        </is>
-      </c>
-      <c r="M29" s="7" t="inlineStr">
-        <is>
-          <t>projects/04-columnar-query-engine/backend/tests/sql_tests.rs</t>
-        </is>
-      </c>
-      <c r="N29" s="7" t="inlineStr">
-        <is>
-          <t>4</t>
-        </is>
-      </c>
+          <t>Specified</t>
+        </is>
+      </c>
+      <c r="M29" s="7" t="inlineStr"/>
+      <c r="N29" s="7" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" s="3" t="n">
@@ -2368,31 +2360,23 @@
           <t>04-032</t>
         </is>
       </c>
-      <c r="J36" s="9" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="K36" s="9" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="J36" s="8" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="K36" s="8" t="inlineStr">
+        <is>
+          <t>✗</t>
         </is>
       </c>
       <c r="L36" s="7" t="inlineStr">
         <is>
-          <t>Verified</t>
-        </is>
-      </c>
-      <c r="M36" s="7" t="inlineStr">
-        <is>
-          <t>projects/04-columnar-query-engine/backend/tests/sql_tests.rs</t>
-        </is>
-      </c>
-      <c r="N36" s="7" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+          <t>Specified</t>
+        </is>
+      </c>
+      <c r="M36" s="7" t="inlineStr"/>
+      <c r="N36" s="7" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" s="3" t="n">
@@ -2426,31 +2410,23 @@
           <t>04-033</t>
         </is>
       </c>
-      <c r="J37" s="9" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="K37" s="9" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="J37" s="8" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="K37" s="8" t="inlineStr">
+        <is>
+          <t>✗</t>
         </is>
       </c>
       <c r="L37" s="7" t="inlineStr">
         <is>
-          <t>Verified</t>
-        </is>
-      </c>
-      <c r="M37" s="7" t="inlineStr">
-        <is>
-          <t>projects/04-columnar-query-engine/backend/tests/sql_tests.rs</t>
-        </is>
-      </c>
-      <c r="N37" s="7" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+          <t>Specified</t>
+        </is>
+      </c>
+      <c r="M37" s="7" t="inlineStr"/>
+      <c r="N37" s="7" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" s="3" t="n">
@@ -2484,31 +2460,23 @@
           <t>04-034</t>
         </is>
       </c>
-      <c r="J38" s="9" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="K38" s="9" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="J38" s="8" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="K38" s="8" t="inlineStr">
+        <is>
+          <t>✗</t>
         </is>
       </c>
       <c r="L38" s="7" t="inlineStr">
         <is>
-          <t>Verified</t>
-        </is>
-      </c>
-      <c r="M38" s="7" t="inlineStr">
-        <is>
-          <t>projects/04-columnar-query-engine/backend/tests/sql_tests.rs</t>
-        </is>
-      </c>
-      <c r="N38" s="7" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
-      </c>
+          <t>Specified</t>
+        </is>
+      </c>
+      <c r="M38" s="7" t="inlineStr"/>
+      <c r="N38" s="7" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" s="3" t="n">
@@ -2542,31 +2510,23 @@
           <t>04-035</t>
         </is>
       </c>
-      <c r="J39" s="9" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="K39" s="9" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="J39" s="8" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="K39" s="8" t="inlineStr">
+        <is>
+          <t>✗</t>
         </is>
       </c>
       <c r="L39" s="7" t="inlineStr">
         <is>
-          <t>Verified</t>
-        </is>
-      </c>
-      <c r="M39" s="7" t="inlineStr">
-        <is>
-          <t>projects/04-columnar-query-engine/backend/tests/sql_tests.rs</t>
-        </is>
-      </c>
-      <c r="N39" s="7" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
+          <t>Specified</t>
+        </is>
+      </c>
+      <c r="M39" s="7" t="inlineStr"/>
+      <c r="N39" s="7" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" s="3" t="n">
@@ -4831,12 +4791,12 @@
       </c>
       <c r="M83" s="7" t="inlineStr">
         <is>
-          <t>projects/04-columnar-query-engine/backend/tests/sql_tests.rs</t>
+          <t>projects/04-columnar-query-engine/backend/tests/morsel_tests.rs</t>
         </is>
       </c>
       <c r="N83" s="7" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>3</t>
         </is>
       </c>
     </row>
@@ -4872,23 +4832,31 @@
           <t>04-080</t>
         </is>
       </c>
-      <c r="J84" s="8" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="K84" s="8" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="J84" s="9" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="K84" s="9" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="L84" s="7" t="inlineStr">
         <is>
-          <t>Specified</t>
-        </is>
-      </c>
-      <c r="M84" s="7" t="inlineStr"/>
-      <c r="N84" s="7" t="inlineStr"/>
+          <t>Verified</t>
+        </is>
+      </c>
+      <c r="M84" s="7" t="inlineStr">
+        <is>
+          <t>projects/04-columnar-query-engine/backend/tests/morsel_tests.rs</t>
+        </is>
+      </c>
+      <c r="N84" s="7" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
     </row>
     <row r="85">
       <c r="A85" s="3" t="n">
@@ -4922,23 +4890,31 @@
           <t>04-081</t>
         </is>
       </c>
-      <c r="J85" s="8" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="K85" s="8" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="J85" s="9" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="K85" s="9" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="L85" s="7" t="inlineStr">
         <is>
-          <t>Specified</t>
-        </is>
-      </c>
-      <c r="M85" s="7" t="inlineStr"/>
-      <c r="N85" s="7" t="inlineStr"/>
+          <t>Verified</t>
+        </is>
+      </c>
+      <c r="M85" s="7" t="inlineStr">
+        <is>
+          <t>projects/04-columnar-query-engine/backend/tests/morsel_tests.rs</t>
+        </is>
+      </c>
+      <c r="N85" s="7" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
     </row>
     <row r="86">
       <c r="A86" s="3" t="n">
@@ -4972,23 +4948,31 @@
           <t>04-082</t>
         </is>
       </c>
-      <c r="J86" s="8" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="K86" s="8" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="J86" s="9" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="K86" s="9" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="L86" s="7" t="inlineStr">
         <is>
-          <t>Specified</t>
-        </is>
-      </c>
-      <c r="M86" s="7" t="inlineStr"/>
-      <c r="N86" s="7" t="inlineStr"/>
+          <t>Verified</t>
+        </is>
+      </c>
+      <c r="M86" s="7" t="inlineStr">
+        <is>
+          <t>projects/04-columnar-query-engine/backend/tests/morsel_tests.rs</t>
+        </is>
+      </c>
+      <c r="N86" s="7" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
     </row>
     <row r="87">
       <c r="A87" s="3" t="n">
@@ -5022,23 +5006,31 @@
           <t>04-083</t>
         </is>
       </c>
-      <c r="J87" s="8" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="K87" s="8" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="J87" s="9" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="K87" s="9" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="L87" s="7" t="inlineStr">
         <is>
-          <t>Specified</t>
-        </is>
-      </c>
-      <c r="M87" s="7" t="inlineStr"/>
-      <c r="N87" s="7" t="inlineStr"/>
+          <t>Verified</t>
+        </is>
+      </c>
+      <c r="M87" s="7" t="inlineStr">
+        <is>
+          <t>projects/04-columnar-query-engine/backend/tests/morsel_tests.rs</t>
+        </is>
+      </c>
+      <c r="N87" s="7" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
     </row>
     <row r="88">
       <c r="A88" s="3" t="n">
@@ -5072,23 +5064,31 @@
           <t>04-084</t>
         </is>
       </c>
-      <c r="J88" s="8" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="K88" s="8" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="J88" s="9" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="K88" s="9" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="L88" s="7" t="inlineStr">
         <is>
-          <t>Specified</t>
-        </is>
-      </c>
-      <c r="M88" s="7" t="inlineStr"/>
-      <c r="N88" s="7" t="inlineStr"/>
+          <t>Verified</t>
+        </is>
+      </c>
+      <c r="M88" s="7" t="inlineStr">
+        <is>
+          <t>projects/04-columnar-query-engine/backend/tests/morsel_tests.rs</t>
+        </is>
+      </c>
+      <c r="N88" s="7" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
     </row>
     <row r="89">
       <c r="A89" s="3" t="n">
@@ -5122,23 +5122,31 @@
           <t>04-085</t>
         </is>
       </c>
-      <c r="J89" s="8" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="K89" s="8" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="J89" s="9" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="K89" s="9" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="L89" s="7" t="inlineStr">
         <is>
-          <t>Specified</t>
-        </is>
-      </c>
-      <c r="M89" s="7" t="inlineStr"/>
-      <c r="N89" s="7" t="inlineStr"/>
+          <t>Verified</t>
+        </is>
+      </c>
+      <c r="M89" s="7" t="inlineStr">
+        <is>
+          <t>projects/04-columnar-query-engine/backend/tests/morsel_tests.rs</t>
+        </is>
+      </c>
+      <c r="N89" s="7" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
     </row>
     <row r="90">
       <c r="A90" s="3" t="n">
@@ -10334,31 +10342,23 @@
           <t>04-025</t>
         </is>
       </c>
-      <c r="O26" s="9" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="P26" s="9" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="O26" s="8" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="P26" s="8" t="inlineStr">
+        <is>
+          <t>✗</t>
         </is>
       </c>
       <c r="Q26" s="7" t="inlineStr">
         <is>
-          <t>Verified</t>
-        </is>
-      </c>
-      <c r="R26" s="7" t="inlineStr">
-        <is>
-          <t>projects/04-columnar-query-engine/backend/tests/sql_tests.rs</t>
-        </is>
-      </c>
-      <c r="S26" s="7" t="inlineStr">
-        <is>
-          <t>4</t>
-        </is>
-      </c>
+          <t>Specified</t>
+        </is>
+      </c>
+      <c r="R26" s="7" t="inlineStr"/>
+      <c r="S26" s="7" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" s="5" t="n">
@@ -10869,31 +10869,23 @@
           <t>04-032</t>
         </is>
       </c>
-      <c r="O33" s="9" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="P33" s="9" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="O33" s="8" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="P33" s="8" t="inlineStr">
+        <is>
+          <t>✗</t>
         </is>
       </c>
       <c r="Q33" s="7" t="inlineStr">
         <is>
-          <t>Verified</t>
-        </is>
-      </c>
-      <c r="R33" s="7" t="inlineStr">
-        <is>
-          <t>projects/04-columnar-query-engine/backend/tests/sql_tests.rs</t>
-        </is>
-      </c>
-      <c r="S33" s="7" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+          <t>Specified</t>
+        </is>
+      </c>
+      <c r="R33" s="7" t="inlineStr"/>
+      <c r="S33" s="7" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" s="5" t="n">
@@ -10950,31 +10942,23 @@
           <t>04-033</t>
         </is>
       </c>
-      <c r="O34" s="9" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="P34" s="9" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="O34" s="8" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="P34" s="8" t="inlineStr">
+        <is>
+          <t>✗</t>
         </is>
       </c>
       <c r="Q34" s="7" t="inlineStr">
         <is>
-          <t>Verified</t>
-        </is>
-      </c>
-      <c r="R34" s="7" t="inlineStr">
-        <is>
-          <t>projects/04-columnar-query-engine/backend/tests/sql_tests.rs</t>
-        </is>
-      </c>
-      <c r="S34" s="7" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+          <t>Specified</t>
+        </is>
+      </c>
+      <c r="R34" s="7" t="inlineStr"/>
+      <c r="S34" s="7" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" s="5" t="n">
@@ -11031,31 +11015,23 @@
           <t>04-034</t>
         </is>
       </c>
-      <c r="O35" s="9" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="P35" s="9" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="O35" s="8" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="P35" s="8" t="inlineStr">
+        <is>
+          <t>✗</t>
         </is>
       </c>
       <c r="Q35" s="7" t="inlineStr">
         <is>
-          <t>Verified</t>
-        </is>
-      </c>
-      <c r="R35" s="7" t="inlineStr">
-        <is>
-          <t>projects/04-columnar-query-engine/backend/tests/sql_tests.rs</t>
-        </is>
-      </c>
-      <c r="S35" s="7" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
-      </c>
+          <t>Specified</t>
+        </is>
+      </c>
+      <c r="R35" s="7" t="inlineStr"/>
+      <c r="S35" s="7" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" s="5" t="n">
@@ -11112,31 +11088,23 @@
           <t>04-035</t>
         </is>
       </c>
-      <c r="O36" s="9" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="P36" s="9" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="O36" s="8" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="P36" s="8" t="inlineStr">
+        <is>
+          <t>✗</t>
         </is>
       </c>
       <c r="Q36" s="7" t="inlineStr">
         <is>
-          <t>Verified</t>
-        </is>
-      </c>
-      <c r="R36" s="7" t="inlineStr">
-        <is>
-          <t>projects/04-columnar-query-engine/backend/tests/sql_tests.rs</t>
-        </is>
-      </c>
-      <c r="S36" s="7" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
+          <t>Specified</t>
+        </is>
+      </c>
+      <c r="R36" s="7" t="inlineStr"/>
+      <c r="S36" s="7" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" s="5" t="n">
@@ -14413,12 +14381,12 @@
       </c>
       <c r="R80" s="7" t="inlineStr">
         <is>
-          <t>projects/04-columnar-query-engine/backend/tests/sql_tests.rs</t>
+          <t>projects/04-columnar-query-engine/backend/tests/morsel_tests.rs</t>
         </is>
       </c>
       <c r="S80" s="7" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>3</t>
         </is>
       </c>
     </row>
@@ -14477,23 +14445,31 @@
           <t>04-080</t>
         </is>
       </c>
-      <c r="O81" s="8" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="P81" s="8" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="O81" s="9" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="P81" s="9" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="Q81" s="7" t="inlineStr">
         <is>
-          <t>Specified</t>
-        </is>
-      </c>
-      <c r="R81" s="7" t="inlineStr"/>
-      <c r="S81" s="7" t="inlineStr"/>
+          <t>Verified</t>
+        </is>
+      </c>
+      <c r="R81" s="7" t="inlineStr">
+        <is>
+          <t>projects/04-columnar-query-engine/backend/tests/morsel_tests.rs</t>
+        </is>
+      </c>
+      <c r="S81" s="7" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
     </row>
     <row r="82">
       <c r="A82" s="5" t="n">
@@ -14550,23 +14526,31 @@
           <t>04-081</t>
         </is>
       </c>
-      <c r="O82" s="8" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="P82" s="8" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="O82" s="9" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="P82" s="9" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="Q82" s="7" t="inlineStr">
         <is>
-          <t>Specified</t>
-        </is>
-      </c>
-      <c r="R82" s="7" t="inlineStr"/>
-      <c r="S82" s="7" t="inlineStr"/>
+          <t>Verified</t>
+        </is>
+      </c>
+      <c r="R82" s="7" t="inlineStr">
+        <is>
+          <t>projects/04-columnar-query-engine/backend/tests/morsel_tests.rs</t>
+        </is>
+      </c>
+      <c r="S82" s="7" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
     </row>
     <row r="83">
       <c r="A83" s="5" t="n">
@@ -14623,23 +14607,31 @@
           <t>04-082</t>
         </is>
       </c>
-      <c r="O83" s="8" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="P83" s="8" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="O83" s="9" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="P83" s="9" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="Q83" s="7" t="inlineStr">
         <is>
-          <t>Specified</t>
-        </is>
-      </c>
-      <c r="R83" s="7" t="inlineStr"/>
-      <c r="S83" s="7" t="inlineStr"/>
+          <t>Verified</t>
+        </is>
+      </c>
+      <c r="R83" s="7" t="inlineStr">
+        <is>
+          <t>projects/04-columnar-query-engine/backend/tests/morsel_tests.rs</t>
+        </is>
+      </c>
+      <c r="S83" s="7" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
     </row>
     <row r="84">
       <c r="A84" s="5" t="n">
@@ -14696,23 +14688,31 @@
           <t>04-083</t>
         </is>
       </c>
-      <c r="O84" s="8" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="P84" s="8" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="O84" s="9" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="P84" s="9" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="Q84" s="7" t="inlineStr">
         <is>
-          <t>Specified</t>
-        </is>
-      </c>
-      <c r="R84" s="7" t="inlineStr"/>
-      <c r="S84" s="7" t="inlineStr"/>
+          <t>Verified</t>
+        </is>
+      </c>
+      <c r="R84" s="7" t="inlineStr">
+        <is>
+          <t>projects/04-columnar-query-engine/backend/tests/morsel_tests.rs</t>
+        </is>
+      </c>
+      <c r="S84" s="7" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
     </row>
     <row r="85">
       <c r="A85" s="5" t="n">
@@ -14769,23 +14769,31 @@
           <t>04-084</t>
         </is>
       </c>
-      <c r="O85" s="8" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="P85" s="8" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="O85" s="9" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="P85" s="9" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="Q85" s="7" t="inlineStr">
         <is>
-          <t>Specified</t>
-        </is>
-      </c>
-      <c r="R85" s="7" t="inlineStr"/>
-      <c r="S85" s="7" t="inlineStr"/>
+          <t>Verified</t>
+        </is>
+      </c>
+      <c r="R85" s="7" t="inlineStr">
+        <is>
+          <t>projects/04-columnar-query-engine/backend/tests/morsel_tests.rs</t>
+        </is>
+      </c>
+      <c r="S85" s="7" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
     </row>
     <row r="86">
       <c r="A86" s="5" t="n">
@@ -14842,23 +14850,31 @@
           <t>04-085</t>
         </is>
       </c>
-      <c r="O86" s="8" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="P86" s="8" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="O86" s="9" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="P86" s="9" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="Q86" s="7" t="inlineStr">
         <is>
-          <t>Specified</t>
-        </is>
-      </c>
-      <c r="R86" s="7" t="inlineStr"/>
-      <c r="S86" s="7" t="inlineStr"/>
+          <t>Verified</t>
+        </is>
+      </c>
+      <c r="R86" s="7" t="inlineStr">
+        <is>
+          <t>projects/04-columnar-query-engine/backend/tests/morsel_tests.rs</t>
+        </is>
+      </c>
+      <c r="S86" s="7" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
     </row>
     <row r="87">
       <c r="A87" s="5" t="n">
@@ -20095,7 +20111,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-10-01 21:18:35</t>
+          <t>2026-10-01 22:59:51</t>
         </is>
       </c>
     </row>
@@ -20107,7 +20123,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>49adde6</t>
+          <t>e04913e</t>
         </is>
       </c>
     </row>
@@ -20381,26 +20397,22 @@
           <t>P0</t>
         </is>
       </c>
-      <c r="D16" s="9" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="E16" s="9" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="D16" s="8" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="E16" s="8" t="inlineStr">
+        <is>
+          <t>✗</t>
         </is>
       </c>
       <c r="F16" s="7" t="inlineStr">
         <is>
-          <t>Verified</t>
-        </is>
-      </c>
-      <c r="G16" s="7" t="inlineStr">
-        <is>
-          <t>projects/04-columnar-query-engine/backend/tests/sql_tests.rs</t>
-        </is>
-      </c>
+          <t>Specified</t>
+        </is>
+      </c>
+      <c r="G16" s="7" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" s="7" t="inlineStr">
@@ -20492,26 +20504,22 @@
           <t>P0</t>
         </is>
       </c>
-      <c r="D19" s="9" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="E19" s="9" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="D19" s="8" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="E19" s="8" t="inlineStr">
+        <is>
+          <t>✗</t>
         </is>
       </c>
       <c r="F19" s="7" t="inlineStr">
         <is>
-          <t>Verified</t>
-        </is>
-      </c>
-      <c r="G19" s="7" t="inlineStr">
-        <is>
-          <t>projects/04-columnar-query-engine/backend/tests/sql_tests.rs</t>
-        </is>
-      </c>
+          <t>Specified</t>
+        </is>
+      </c>
+      <c r="G19" s="7" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" s="7" t="inlineStr">
@@ -20529,26 +20537,22 @@
           <t>P0</t>
         </is>
       </c>
-      <c r="D20" s="9" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="E20" s="9" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="D20" s="8" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="E20" s="8" t="inlineStr">
+        <is>
+          <t>✗</t>
         </is>
       </c>
       <c r="F20" s="7" t="inlineStr">
         <is>
-          <t>Verified</t>
-        </is>
-      </c>
-      <c r="G20" s="7" t="inlineStr">
-        <is>
-          <t>projects/04-columnar-query-engine/backend/tests/sql_tests.rs</t>
-        </is>
-      </c>
+          <t>Specified</t>
+        </is>
+      </c>
+      <c r="G20" s="7" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" s="7" t="inlineStr">
@@ -20566,26 +20570,22 @@
           <t>P0</t>
         </is>
       </c>
-      <c r="D21" s="9" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="E21" s="9" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="D21" s="8" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="E21" s="8" t="inlineStr">
+        <is>
+          <t>✗</t>
         </is>
       </c>
       <c r="F21" s="7" t="inlineStr">
         <is>
-          <t>Verified</t>
-        </is>
-      </c>
-      <c r="G21" s="7" t="inlineStr">
-        <is>
-          <t>projects/04-columnar-query-engine/backend/tests/sql_tests.rs</t>
-        </is>
-      </c>
+          <t>Specified</t>
+        </is>
+      </c>
+      <c r="G21" s="7" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" s="7" t="inlineStr">
@@ -20603,26 +20603,22 @@
           <t>P0</t>
         </is>
       </c>
-      <c r="D22" s="9" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="E22" s="9" t="inlineStr">
-        <is>
-          <t>✓</t>
+      <c r="D22" s="8" t="inlineStr">
+        <is>
+          <t>✗</t>
+        </is>
+      </c>
+      <c r="E22" s="8" t="inlineStr">
+        <is>
+          <t>✗</t>
         </is>
       </c>
       <c r="F22" s="7" t="inlineStr">
         <is>
-          <t>Verified</t>
-        </is>
-      </c>
-      <c r="G22" s="7" t="inlineStr">
-        <is>
-          <t>projects/04-columnar-query-engine/backend/tests/sql_tests.rs</t>
-        </is>
-      </c>
+          <t>Specified</t>
+        </is>
+      </c>
+      <c r="G22" s="7" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" s="7" t="inlineStr">
@@ -21349,7 +21345,7 @@
       </c>
       <c r="G43" s="7" t="inlineStr">
         <is>
-          <t>projects/04-columnar-query-engine/backend/tests/sql_tests.rs</t>
+          <t>projects/04-columnar-query-engine/backend/tests/morsel_tests.rs</t>
         </is>
       </c>
     </row>
@@ -21369,22 +21365,26 @@
           <t>P0</t>
         </is>
       </c>
-      <c r="D44" s="8" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="E44" s="8" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="D44" s="9" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="E44" s="9" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="F44" s="7" t="inlineStr">
         <is>
-          <t>Specified</t>
-        </is>
-      </c>
-      <c r="G44" s="7" t="inlineStr"/>
+          <t>Verified</t>
+        </is>
+      </c>
+      <c r="G44" s="7" t="inlineStr">
+        <is>
+          <t>projects/04-columnar-query-engine/backend/tests/morsel_tests.rs</t>
+        </is>
+      </c>
     </row>
     <row r="45">
       <c r="A45" s="7" t="inlineStr">
@@ -21402,22 +21402,26 @@
           <t>P0</t>
         </is>
       </c>
-      <c r="D45" s="8" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="E45" s="8" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="D45" s="9" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="E45" s="9" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="F45" s="7" t="inlineStr">
         <is>
-          <t>Specified</t>
-        </is>
-      </c>
-      <c r="G45" s="7" t="inlineStr"/>
+          <t>Verified</t>
+        </is>
+      </c>
+      <c r="G45" s="7" t="inlineStr">
+        <is>
+          <t>projects/04-columnar-query-engine/backend/tests/morsel_tests.rs</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="A46" s="7" t="inlineStr">
@@ -21435,22 +21439,26 @@
           <t>P0</t>
         </is>
       </c>
-      <c r="D46" s="8" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="E46" s="8" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="D46" s="9" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="E46" s="9" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="F46" s="7" t="inlineStr">
         <is>
-          <t>Specified</t>
-        </is>
-      </c>
-      <c r="G46" s="7" t="inlineStr"/>
+          <t>Verified</t>
+        </is>
+      </c>
+      <c r="G46" s="7" t="inlineStr">
+        <is>
+          <t>projects/04-columnar-query-engine/backend/tests/morsel_tests.rs</t>
+        </is>
+      </c>
     </row>
     <row r="47">
       <c r="A47" s="7" t="inlineStr">
@@ -21468,22 +21476,26 @@
           <t>P0</t>
         </is>
       </c>
-      <c r="D47" s="8" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="E47" s="8" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="D47" s="9" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="E47" s="9" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="F47" s="7" t="inlineStr">
         <is>
-          <t>Specified</t>
-        </is>
-      </c>
-      <c r="G47" s="7" t="inlineStr"/>
+          <t>Verified</t>
+        </is>
+      </c>
+      <c r="G47" s="7" t="inlineStr">
+        <is>
+          <t>projects/04-columnar-query-engine/backend/tests/morsel_tests.rs</t>
+        </is>
+      </c>
     </row>
     <row r="48">
       <c r="A48" s="7" t="inlineStr">
@@ -21501,22 +21513,26 @@
           <t>P0</t>
         </is>
       </c>
-      <c r="D48" s="8" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="E48" s="8" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="D48" s="9" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="E48" s="9" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="F48" s="7" t="inlineStr">
         <is>
-          <t>Specified</t>
-        </is>
-      </c>
-      <c r="G48" s="7" t="inlineStr"/>
+          <t>Verified</t>
+        </is>
+      </c>
+      <c r="G48" s="7" t="inlineStr">
+        <is>
+          <t>projects/04-columnar-query-engine/backend/tests/morsel_tests.rs</t>
+        </is>
+      </c>
     </row>
     <row r="49">
       <c r="A49" s="7" t="inlineStr">
@@ -21534,22 +21550,26 @@
           <t>P0</t>
         </is>
       </c>
-      <c r="D49" s="8" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="E49" s="8" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="D49" s="9" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="E49" s="9" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="F49" s="7" t="inlineStr">
         <is>
-          <t>Specified</t>
-        </is>
-      </c>
-      <c r="G49" s="7" t="inlineStr"/>
+          <t>Verified</t>
+        </is>
+      </c>
+      <c r="G49" s="7" t="inlineStr">
+        <is>
+          <t>projects/04-columnar-query-engine/backend/tests/morsel_tests.rs</t>
+        </is>
+      </c>
     </row>
     <row r="50">
       <c r="A50" s="7" t="inlineStr">

</xml_diff>

<commit_message>
S10 Part 0: Carry-over integrity, hash checks, count consistency gate, and deferred verification register
</commit_message>
<xml_diff>
--- a/evidence/workbooks/04_Columnar_Query_Engine_ULTIMATE_145_Master_STATUS.xlsx
+++ b/evidence/workbooks/04_Columnar_Query_Engine_ULTIMATE_145_Master_STATUS.xlsx
@@ -2116,7 +2116,7 @@
       </c>
       <c r="N31" s="7" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>5</t>
         </is>
       </c>
     </row>
@@ -2174,7 +2174,7 @@
       </c>
       <c r="N32" s="7" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>4</t>
         </is>
       </c>
     </row>
@@ -2782,7 +2782,7 @@
       </c>
       <c r="N44" s="7" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3</t>
         </is>
       </c>
     </row>
@@ -2840,7 +2840,7 @@
       </c>
       <c r="N45" s="7" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>3</t>
         </is>
       </c>
     </row>
@@ -4796,7 +4796,7 @@
       </c>
       <c r="N83" s="7" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>8</t>
         </is>
       </c>
     </row>
@@ -4854,7 +4854,7 @@
       </c>
       <c r="N84" s="7" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>5</t>
         </is>
       </c>
     </row>
@@ -4970,7 +4970,7 @@
       </c>
       <c r="N86" s="7" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>5</t>
         </is>
       </c>
     </row>
@@ -5028,7 +5028,7 @@
       </c>
       <c r="N87" s="7" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>7</t>
         </is>
       </c>
     </row>
@@ -10510,7 +10510,7 @@
       </c>
       <c r="S28" s="7" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>5</t>
         </is>
       </c>
     </row>
@@ -10591,7 +10591,7 @@
       </c>
       <c r="S29" s="7" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>4</t>
         </is>
       </c>
     </row>
@@ -11475,7 +11475,7 @@
       </c>
       <c r="S41" s="7" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3</t>
         </is>
       </c>
     </row>
@@ -11556,7 +11556,7 @@
       </c>
       <c r="S42" s="7" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>3</t>
         </is>
       </c>
     </row>
@@ -14386,7 +14386,7 @@
       </c>
       <c r="S80" s="7" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>8</t>
         </is>
       </c>
     </row>
@@ -14467,7 +14467,7 @@
       </c>
       <c r="S81" s="7" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>5</t>
         </is>
       </c>
     </row>
@@ -14629,7 +14629,7 @@
       </c>
       <c r="S83" s="7" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>5</t>
         </is>
       </c>
     </row>
@@ -14710,7 +14710,7 @@
       </c>
       <c r="S84" s="7" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>7</t>
         </is>
       </c>
     </row>
@@ -20111,7 +20111,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-10-01 22:59:51</t>
+          <t>2026-10-02 10:31:41</t>
         </is>
       </c>
     </row>
@@ -20123,7 +20123,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>e04913e</t>
+          <t>80489b0</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
S10 Part 1: Mini-QUIC in-tree TLS 1.3 handshake, real interop corpus with aioquic, UDP loopback integration, and security P0 batch
</commit_message>
<xml_diff>
--- a/evidence/workbooks/04_Columnar_Query_Engine_ULTIMATE_145_Master_STATUS.xlsx
+++ b/evidence/workbooks/04_Columnar_Query_Engine_ULTIMATE_145_Master_STATUS.xlsx
@@ -20111,7 +20111,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-10-02 10:31:41</t>
+          <t>2026-10-02 10:41:41</t>
         </is>
       </c>
     </row>
@@ -20123,7 +20123,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>80489b0</t>
+          <t>e20d5f2</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
S10 Part 2: 06 LSM Spine unified engine path, snapshot isolation, multi-level scan, WAL rotation, group commit, and crash consistency
</commit_message>
<xml_diff>
--- a/evidence/workbooks/04_Columnar_Query_Engine_ULTIMATE_145_Master_STATUS.xlsx
+++ b/evidence/workbooks/04_Columnar_Query_Engine_ULTIMATE_145_Master_STATUS.xlsx
@@ -20111,7 +20111,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-10-02 10:41:41</t>
+          <t>2026-10-02 10:43:55</t>
         </is>
       </c>
     </row>
@@ -20123,7 +20123,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>e20d5f2</t>
+          <t>153705e</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
S10 Part 3: 04 Columnar SQL execution depth, NULL semantics, differential DuckDB tests, TPC-H SF1, and query optimization
</commit_message>
<xml_diff>
--- a/evidence/workbooks/04_Columnar_Query_Engine_ULTIMATE_145_Master_STATUS.xlsx
+++ b/evidence/workbooks/04_Columnar_Query_Engine_ULTIMATE_145_Master_STATUS.xlsx
@@ -1994,23 +1994,31 @@
           <t>04-025</t>
         </is>
       </c>
-      <c r="J29" s="8" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="K29" s="8" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="J29" s="9" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="K29" s="9" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="L29" s="7" t="inlineStr">
         <is>
-          <t>Specified</t>
-        </is>
-      </c>
-      <c r="M29" s="7" t="inlineStr"/>
-      <c r="N29" s="7" t="inlineStr"/>
+          <t>Verified</t>
+        </is>
+      </c>
+      <c r="M29" s="7" t="inlineStr">
+        <is>
+          <t>projects/04-columnar-query-engine/backend/tests/sql_tests.rs</t>
+        </is>
+      </c>
+      <c r="N29" s="7" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="3" t="n">
@@ -2360,23 +2368,31 @@
           <t>04-032</t>
         </is>
       </c>
-      <c r="J36" s="8" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="K36" s="8" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="J36" s="9" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="K36" s="9" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="L36" s="7" t="inlineStr">
         <is>
-          <t>Specified</t>
-        </is>
-      </c>
-      <c r="M36" s="7" t="inlineStr"/>
-      <c r="N36" s="7" t="inlineStr"/>
+          <t>Verified</t>
+        </is>
+      </c>
+      <c r="M36" s="7" t="inlineStr">
+        <is>
+          <t>projects/04-columnar-query-engine/backend/tests/sql_tests.rs</t>
+        </is>
+      </c>
+      <c r="N36" s="7" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="3" t="n">
@@ -2410,23 +2426,31 @@
           <t>04-033</t>
         </is>
       </c>
-      <c r="J37" s="8" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="K37" s="8" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="J37" s="9" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="K37" s="9" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="L37" s="7" t="inlineStr">
         <is>
-          <t>Specified</t>
-        </is>
-      </c>
-      <c r="M37" s="7" t="inlineStr"/>
-      <c r="N37" s="7" t="inlineStr"/>
+          <t>Verified</t>
+        </is>
+      </c>
+      <c r="M37" s="7" t="inlineStr">
+        <is>
+          <t>projects/04-columnar-query-engine/backend/tests/sql_tests.rs</t>
+        </is>
+      </c>
+      <c r="N37" s="7" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="3" t="n">
@@ -2460,23 +2484,31 @@
           <t>04-034</t>
         </is>
       </c>
-      <c r="J38" s="8" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="K38" s="8" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="J38" s="9" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="K38" s="9" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="L38" s="7" t="inlineStr">
         <is>
-          <t>Specified</t>
-        </is>
-      </c>
-      <c r="M38" s="7" t="inlineStr"/>
-      <c r="N38" s="7" t="inlineStr"/>
+          <t>Verified</t>
+        </is>
+      </c>
+      <c r="M38" s="7" t="inlineStr">
+        <is>
+          <t>projects/04-columnar-query-engine/backend/tests/sql_tests.rs</t>
+        </is>
+      </c>
+      <c r="N38" s="7" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="3" t="n">
@@ -2510,23 +2542,31 @@
           <t>04-035</t>
         </is>
       </c>
-      <c r="J39" s="8" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="K39" s="8" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="J39" s="9" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="K39" s="9" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="L39" s="7" t="inlineStr">
         <is>
-          <t>Specified</t>
-        </is>
-      </c>
-      <c r="M39" s="7" t="inlineStr"/>
-      <c r="N39" s="7" t="inlineStr"/>
+          <t>Verified</t>
+        </is>
+      </c>
+      <c r="M39" s="7" t="inlineStr">
+        <is>
+          <t>projects/04-columnar-query-engine/backend/tests/sql_tests.rs</t>
+        </is>
+      </c>
+      <c r="N39" s="7" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="3" t="n">
@@ -2610,23 +2650,31 @@
           <t>04-037</t>
         </is>
       </c>
-      <c r="J41" s="8" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="K41" s="8" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="J41" s="9" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="K41" s="9" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="L41" s="7" t="inlineStr">
         <is>
-          <t>Specified</t>
-        </is>
-      </c>
-      <c r="M41" s="7" t="inlineStr"/>
-      <c r="N41" s="7" t="inlineStr"/>
+          <t>Verified</t>
+        </is>
+      </c>
+      <c r="M41" s="7" t="inlineStr">
+        <is>
+          <t>projects/04-columnar-query-engine/backend/tests/sql_tests.rs</t>
+        </is>
+      </c>
+      <c r="N41" s="7" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="3" t="n">
@@ -2710,23 +2758,31 @@
           <t>04-039</t>
         </is>
       </c>
-      <c r="J43" s="8" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="K43" s="8" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="J43" s="9" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="K43" s="9" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="L43" s="7" t="inlineStr">
         <is>
-          <t>Specified</t>
-        </is>
-      </c>
-      <c r="M43" s="7" t="inlineStr"/>
-      <c r="N43" s="7" t="inlineStr"/>
+          <t>Verified</t>
+        </is>
+      </c>
+      <c r="M43" s="7" t="inlineStr">
+        <is>
+          <t>projects/04-columnar-query-engine/backend/tests/sql_tests.rs</t>
+        </is>
+      </c>
+      <c r="N43" s="7" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="A44" s="3" t="n">
@@ -2876,23 +2932,31 @@
           <t>04-042</t>
         </is>
       </c>
-      <c r="J46" s="8" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="K46" s="8" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="J46" s="9" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="K46" s="9" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="L46" s="7" t="inlineStr">
         <is>
-          <t>Specified</t>
-        </is>
-      </c>
-      <c r="M46" s="7" t="inlineStr"/>
-      <c r="N46" s="7" t="inlineStr"/>
+          <t>Verified</t>
+        </is>
+      </c>
+      <c r="M46" s="7" t="inlineStr">
+        <is>
+          <t>projects/04-columnar-query-engine/backend/tests/sql_tests.rs</t>
+        </is>
+      </c>
+      <c r="N46" s="7" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
     </row>
     <row r="47">
       <c r="A47" s="3" t="n">
@@ -2926,23 +2990,31 @@
           <t>04-043</t>
         </is>
       </c>
-      <c r="J47" s="8" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="K47" s="8" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="J47" s="9" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="K47" s="9" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="L47" s="7" t="inlineStr">
         <is>
-          <t>Specified</t>
-        </is>
-      </c>
-      <c r="M47" s="7" t="inlineStr"/>
-      <c r="N47" s="7" t="inlineStr"/>
+          <t>Verified</t>
+        </is>
+      </c>
+      <c r="M47" s="7" t="inlineStr">
+        <is>
+          <t>projects/04-columnar-query-engine/backend/tests/sql_tests.rs</t>
+        </is>
+      </c>
+      <c r="N47" s="7" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
     </row>
     <row r="48">
       <c r="A48" s="3" t="n">
@@ -4174,23 +4246,31 @@
           <t>04-067</t>
         </is>
       </c>
-      <c r="J71" s="8" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="K71" s="8" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="J71" s="9" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="K71" s="9" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="L71" s="7" t="inlineStr">
         <is>
-          <t>Specified</t>
-        </is>
-      </c>
-      <c r="M71" s="7" t="inlineStr"/>
-      <c r="N71" s="7" t="inlineStr"/>
+          <t>Verified</t>
+        </is>
+      </c>
+      <c r="M71" s="7" t="inlineStr">
+        <is>
+          <t>projects/04-columnar-query-engine/backend/tests/sql_tests.rs</t>
+        </is>
+      </c>
+      <c r="N71" s="7" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
     </row>
     <row r="72">
       <c r="A72" s="3" t="n">
@@ -5880,23 +5960,31 @@
           <t>04-100</t>
         </is>
       </c>
-      <c r="J104" s="8" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="K104" s="8" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="J104" s="9" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="K104" s="9" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="L104" s="7" t="inlineStr">
         <is>
-          <t>Specified</t>
-        </is>
-      </c>
-      <c r="M104" s="7" t="inlineStr"/>
-      <c r="N104" s="7" t="inlineStr"/>
+          <t>Verified</t>
+        </is>
+      </c>
+      <c r="M104" s="7" t="inlineStr">
+        <is>
+          <t>projects/04-columnar-query-engine/backend/tests/sql_tests.rs</t>
+        </is>
+      </c>
+      <c r="N104" s="7" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
     </row>
     <row r="105">
       <c r="A105" s="3" t="n">
@@ -6084,23 +6172,31 @@
           <t>04-104</t>
         </is>
       </c>
-      <c r="J108" s="8" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="K108" s="8" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="J108" s="9" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="K108" s="9" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="L108" s="7" t="inlineStr">
         <is>
-          <t>Specified</t>
-        </is>
-      </c>
-      <c r="M108" s="7" t="inlineStr"/>
-      <c r="N108" s="7" t="inlineStr"/>
+          <t>Verified</t>
+        </is>
+      </c>
+      <c r="M108" s="7" t="inlineStr">
+        <is>
+          <t>projects/04-columnar-query-engine/backend/tests/sql_tests.rs</t>
+        </is>
+      </c>
+      <c r="N108" s="7" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
     </row>
     <row r="109">
       <c r="A109" s="3" t="n">
@@ -6138,23 +6234,31 @@
           <t>04-105</t>
         </is>
       </c>
-      <c r="J109" s="8" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="K109" s="8" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="J109" s="9" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="K109" s="9" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="L109" s="7" t="inlineStr">
         <is>
-          <t>Specified</t>
-        </is>
-      </c>
-      <c r="M109" s="7" t="inlineStr"/>
-      <c r="N109" s="7" t="inlineStr"/>
+          <t>Verified</t>
+        </is>
+      </c>
+      <c r="M109" s="7" t="inlineStr">
+        <is>
+          <t>projects/04-columnar-query-engine/backend/tests/sql_tests.rs</t>
+        </is>
+      </c>
+      <c r="N109" s="7" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
     </row>
     <row r="110">
       <c r="A110" s="3" t="n">
@@ -7366,23 +7470,31 @@
           <t>04-127</t>
         </is>
       </c>
-      <c r="J131" s="8" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="K131" s="8" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="J131" s="9" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="K131" s="9" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="L131" s="7" t="inlineStr">
         <is>
-          <t>Specified</t>
-        </is>
-      </c>
-      <c r="M131" s="7" t="inlineStr"/>
-      <c r="N131" s="7" t="inlineStr"/>
+          <t>Verified</t>
+        </is>
+      </c>
+      <c r="M131" s="7" t="inlineStr">
+        <is>
+          <t>projects/04-columnar-query-engine/backend/tests/sql_tests.rs</t>
+        </is>
+      </c>
+      <c r="N131" s="7" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
     </row>
     <row r="132">
       <c r="A132" s="3" t="n">
@@ -7716,23 +7828,31 @@
           <t>04-134</t>
         </is>
       </c>
-      <c r="J138" s="8" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="K138" s="8" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="J138" s="9" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="K138" s="9" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="L138" s="7" t="inlineStr">
         <is>
-          <t>Specified</t>
-        </is>
-      </c>
-      <c r="M138" s="7" t="inlineStr"/>
-      <c r="N138" s="7" t="inlineStr"/>
+          <t>Verified</t>
+        </is>
+      </c>
+      <c r="M138" s="7" t="inlineStr">
+        <is>
+          <t>projects/04-columnar-query-engine/backend/tests/sql_tests.rs</t>
+        </is>
+      </c>
+      <c r="N138" s="7" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
     </row>
     <row r="139">
       <c r="A139" s="3" t="n">
@@ -10342,23 +10462,31 @@
           <t>04-025</t>
         </is>
       </c>
-      <c r="O26" s="8" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="P26" s="8" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="O26" s="9" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="P26" s="9" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="Q26" s="7" t="inlineStr">
         <is>
-          <t>Specified</t>
-        </is>
-      </c>
-      <c r="R26" s="7" t="inlineStr"/>
-      <c r="S26" s="7" t="inlineStr"/>
+          <t>Verified</t>
+        </is>
+      </c>
+      <c r="R26" s="7" t="inlineStr">
+        <is>
+          <t>projects/04-columnar-query-engine/backend/tests/sql_tests.rs</t>
+        </is>
+      </c>
+      <c r="S26" s="7" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="5" t="n">
@@ -10869,23 +10997,31 @@
           <t>04-032</t>
         </is>
       </c>
-      <c r="O33" s="8" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="P33" s="8" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="O33" s="9" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="P33" s="9" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="Q33" s="7" t="inlineStr">
         <is>
-          <t>Specified</t>
-        </is>
-      </c>
-      <c r="R33" s="7" t="inlineStr"/>
-      <c r="S33" s="7" t="inlineStr"/>
+          <t>Verified</t>
+        </is>
+      </c>
+      <c r="R33" s="7" t="inlineStr">
+        <is>
+          <t>projects/04-columnar-query-engine/backend/tests/sql_tests.rs</t>
+        </is>
+      </c>
+      <c r="S33" s="7" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="5" t="n">
@@ -10942,23 +11078,31 @@
           <t>04-033</t>
         </is>
       </c>
-      <c r="O34" s="8" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="P34" s="8" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="O34" s="9" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="P34" s="9" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="Q34" s="7" t="inlineStr">
         <is>
-          <t>Specified</t>
-        </is>
-      </c>
-      <c r="R34" s="7" t="inlineStr"/>
-      <c r="S34" s="7" t="inlineStr"/>
+          <t>Verified</t>
+        </is>
+      </c>
+      <c r="R34" s="7" t="inlineStr">
+        <is>
+          <t>projects/04-columnar-query-engine/backend/tests/sql_tests.rs</t>
+        </is>
+      </c>
+      <c r="S34" s="7" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="5" t="n">
@@ -11015,23 +11159,31 @@
           <t>04-034</t>
         </is>
       </c>
-      <c r="O35" s="8" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="P35" s="8" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="O35" s="9" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="P35" s="9" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="Q35" s="7" t="inlineStr">
         <is>
-          <t>Specified</t>
-        </is>
-      </c>
-      <c r="R35" s="7" t="inlineStr"/>
-      <c r="S35" s="7" t="inlineStr"/>
+          <t>Verified</t>
+        </is>
+      </c>
+      <c r="R35" s="7" t="inlineStr">
+        <is>
+          <t>projects/04-columnar-query-engine/backend/tests/sql_tests.rs</t>
+        </is>
+      </c>
+      <c r="S35" s="7" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="5" t="n">
@@ -11088,23 +11240,31 @@
           <t>04-035</t>
         </is>
       </c>
-      <c r="O36" s="8" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="P36" s="8" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="O36" s="9" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="P36" s="9" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="Q36" s="7" t="inlineStr">
         <is>
-          <t>Specified</t>
-        </is>
-      </c>
-      <c r="R36" s="7" t="inlineStr"/>
-      <c r="S36" s="7" t="inlineStr"/>
+          <t>Verified</t>
+        </is>
+      </c>
+      <c r="R36" s="7" t="inlineStr">
+        <is>
+          <t>projects/04-columnar-query-engine/backend/tests/sql_tests.rs</t>
+        </is>
+      </c>
+      <c r="S36" s="7" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="5" t="n">
@@ -11234,23 +11394,31 @@
           <t>04-037</t>
         </is>
       </c>
-      <c r="O38" s="8" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="P38" s="8" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="O38" s="9" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="P38" s="9" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="Q38" s="7" t="inlineStr">
         <is>
-          <t>Specified</t>
-        </is>
-      </c>
-      <c r="R38" s="7" t="inlineStr"/>
-      <c r="S38" s="7" t="inlineStr"/>
+          <t>Verified</t>
+        </is>
+      </c>
+      <c r="R38" s="7" t="inlineStr">
+        <is>
+          <t>projects/04-columnar-query-engine/backend/tests/sql_tests.rs</t>
+        </is>
+      </c>
+      <c r="S38" s="7" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="5" t="n">
@@ -11380,23 +11548,31 @@
           <t>04-039</t>
         </is>
       </c>
-      <c r="O40" s="8" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="P40" s="8" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="O40" s="9" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="P40" s="9" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="Q40" s="7" t="inlineStr">
         <is>
-          <t>Specified</t>
-        </is>
-      </c>
-      <c r="R40" s="7" t="inlineStr"/>
-      <c r="S40" s="7" t="inlineStr"/>
+          <t>Verified</t>
+        </is>
+      </c>
+      <c r="R40" s="7" t="inlineStr">
+        <is>
+          <t>projects/04-columnar-query-engine/backend/tests/sql_tests.rs</t>
+        </is>
+      </c>
+      <c r="S40" s="7" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="5" t="n">
@@ -11615,23 +11791,31 @@
           <t>04-042</t>
         </is>
       </c>
-      <c r="O43" s="8" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="P43" s="8" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="O43" s="9" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="P43" s="9" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="Q43" s="7" t="inlineStr">
         <is>
-          <t>Specified</t>
-        </is>
-      </c>
-      <c r="R43" s="7" t="inlineStr"/>
-      <c r="S43" s="7" t="inlineStr"/>
+          <t>Verified</t>
+        </is>
+      </c>
+      <c r="R43" s="7" t="inlineStr">
+        <is>
+          <t>projects/04-columnar-query-engine/backend/tests/sql_tests.rs</t>
+        </is>
+      </c>
+      <c r="S43" s="7" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="A44" s="5" t="n">
@@ -11688,23 +11872,31 @@
           <t>04-043</t>
         </is>
       </c>
-      <c r="O44" s="8" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="P44" s="8" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="O44" s="9" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="P44" s="9" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="Q44" s="7" t="inlineStr">
         <is>
-          <t>Specified</t>
-        </is>
-      </c>
-      <c r="R44" s="7" t="inlineStr"/>
-      <c r="S44" s="7" t="inlineStr"/>
+          <t>Verified</t>
+        </is>
+      </c>
+      <c r="R44" s="7" t="inlineStr">
+        <is>
+          <t>projects/04-columnar-query-engine/backend/tests/sql_tests.rs</t>
+        </is>
+      </c>
+      <c r="S44" s="7" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
     </row>
     <row r="45">
       <c r="A45" s="5" t="n">
@@ -13488,23 +13680,31 @@
           <t>04-067</t>
         </is>
       </c>
-      <c r="O68" s="8" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="P68" s="8" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="O68" s="9" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="P68" s="9" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="Q68" s="7" t="inlineStr">
         <is>
-          <t>Specified</t>
-        </is>
-      </c>
-      <c r="R68" s="7" t="inlineStr"/>
-      <c r="S68" s="7" t="inlineStr"/>
+          <t>Verified</t>
+        </is>
+      </c>
+      <c r="R68" s="7" t="inlineStr">
+        <is>
+          <t>projects/04-columnar-query-engine/backend/tests/sql_tests.rs</t>
+        </is>
+      </c>
+      <c r="S68" s="7" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
     </row>
     <row r="69">
       <c r="A69" s="5" t="n">
@@ -15953,23 +16153,31 @@
           <t>04-100</t>
         </is>
       </c>
-      <c r="O101" s="8" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="P101" s="8" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="O101" s="9" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="P101" s="9" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="Q101" s="7" t="inlineStr">
         <is>
-          <t>Specified</t>
-        </is>
-      </c>
-      <c r="R101" s="7" t="inlineStr"/>
-      <c r="S101" s="7" t="inlineStr"/>
+          <t>Verified</t>
+        </is>
+      </c>
+      <c r="R101" s="7" t="inlineStr">
+        <is>
+          <t>projects/04-columnar-query-engine/backend/tests/sql_tests.rs</t>
+        </is>
+      </c>
+      <c r="S101" s="7" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
     </row>
     <row r="102">
       <c r="A102" s="5" t="n">
@@ -16249,23 +16457,31 @@
           <t>04-104</t>
         </is>
       </c>
-      <c r="O105" s="8" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="P105" s="8" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="O105" s="9" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="P105" s="9" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="Q105" s="7" t="inlineStr">
         <is>
-          <t>Specified</t>
-        </is>
-      </c>
-      <c r="R105" s="7" t="inlineStr"/>
-      <c r="S105" s="7" t="inlineStr"/>
+          <t>Verified</t>
+        </is>
+      </c>
+      <c r="R105" s="7" t="inlineStr">
+        <is>
+          <t>projects/04-columnar-query-engine/backend/tests/sql_tests.rs</t>
+        </is>
+      </c>
+      <c r="S105" s="7" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
     </row>
     <row r="106">
       <c r="A106" s="5" t="n">
@@ -16326,23 +16542,31 @@
           <t>04-105</t>
         </is>
       </c>
-      <c r="O106" s="8" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="P106" s="8" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="O106" s="9" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="P106" s="9" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="Q106" s="7" t="inlineStr">
         <is>
-          <t>Specified</t>
-        </is>
-      </c>
-      <c r="R106" s="7" t="inlineStr"/>
-      <c r="S106" s="7" t="inlineStr"/>
+          <t>Verified</t>
+        </is>
+      </c>
+      <c r="R106" s="7" t="inlineStr">
+        <is>
+          <t>projects/04-columnar-query-engine/backend/tests/sql_tests.rs</t>
+        </is>
+      </c>
+      <c r="S106" s="7" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
     </row>
     <row r="107">
       <c r="A107" s="5" t="n">
@@ -18060,23 +18284,31 @@
           <t>04-127</t>
         </is>
       </c>
-      <c r="O128" s="8" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="P128" s="8" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="O128" s="9" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="P128" s="9" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="Q128" s="7" t="inlineStr">
         <is>
-          <t>Specified</t>
-        </is>
-      </c>
-      <c r="R128" s="7" t="inlineStr"/>
-      <c r="S128" s="7" t="inlineStr"/>
+          <t>Verified</t>
+        </is>
+      </c>
+      <c r="R128" s="7" t="inlineStr">
+        <is>
+          <t>projects/04-columnar-query-engine/backend/tests/sql_tests.rs</t>
+        </is>
+      </c>
+      <c r="S128" s="7" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
     </row>
     <row r="129">
       <c r="A129" s="5" t="n">
@@ -18571,23 +18803,31 @@
           <t>04-134</t>
         </is>
       </c>
-      <c r="O135" s="8" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="P135" s="8" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="O135" s="9" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="P135" s="9" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="Q135" s="7" t="inlineStr">
         <is>
-          <t>Specified</t>
-        </is>
-      </c>
-      <c r="R135" s="7" t="inlineStr"/>
-      <c r="S135" s="7" t="inlineStr"/>
+          <t>Verified</t>
+        </is>
+      </c>
+      <c r="R135" s="7" t="inlineStr">
+        <is>
+          <t>projects/04-columnar-query-engine/backend/tests/sql_tests.rs</t>
+        </is>
+      </c>
+      <c r="S135" s="7" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
     </row>
     <row r="136">
       <c r="A136" s="5" t="n">
@@ -20111,7 +20351,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-10-02 10:43:55</t>
+          <t>2026-10-02 10:47:50</t>
         </is>
       </c>
     </row>
@@ -20123,7 +20363,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>153705e</t>
+          <t>c955892</t>
         </is>
       </c>
     </row>
@@ -20397,22 +20637,26 @@
           <t>P0</t>
         </is>
       </c>
-      <c r="D16" s="8" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="E16" s="8" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="D16" s="9" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="E16" s="9" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="F16" s="7" t="inlineStr">
         <is>
-          <t>Specified</t>
-        </is>
-      </c>
-      <c r="G16" s="7" t="inlineStr"/>
+          <t>Verified</t>
+        </is>
+      </c>
+      <c r="G16" s="7" t="inlineStr">
+        <is>
+          <t>projects/04-columnar-query-engine/backend/tests/sql_tests.rs</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="7" t="inlineStr">
@@ -20504,22 +20748,26 @@
           <t>P0</t>
         </is>
       </c>
-      <c r="D19" s="8" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="E19" s="8" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="D19" s="9" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="E19" s="9" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="F19" s="7" t="inlineStr">
         <is>
-          <t>Specified</t>
-        </is>
-      </c>
-      <c r="G19" s="7" t="inlineStr"/>
+          <t>Verified</t>
+        </is>
+      </c>
+      <c r="G19" s="7" t="inlineStr">
+        <is>
+          <t>projects/04-columnar-query-engine/backend/tests/sql_tests.rs</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="7" t="inlineStr">
@@ -20537,22 +20785,26 @@
           <t>P0</t>
         </is>
       </c>
-      <c r="D20" s="8" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="E20" s="8" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="D20" s="9" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="E20" s="9" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="F20" s="7" t="inlineStr">
         <is>
-          <t>Specified</t>
-        </is>
-      </c>
-      <c r="G20" s="7" t="inlineStr"/>
+          <t>Verified</t>
+        </is>
+      </c>
+      <c r="G20" s="7" t="inlineStr">
+        <is>
+          <t>projects/04-columnar-query-engine/backend/tests/sql_tests.rs</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="7" t="inlineStr">
@@ -20570,22 +20822,26 @@
           <t>P0</t>
         </is>
       </c>
-      <c r="D21" s="8" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="E21" s="8" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="D21" s="9" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="E21" s="9" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="F21" s="7" t="inlineStr">
         <is>
-          <t>Specified</t>
-        </is>
-      </c>
-      <c r="G21" s="7" t="inlineStr"/>
+          <t>Verified</t>
+        </is>
+      </c>
+      <c r="G21" s="7" t="inlineStr">
+        <is>
+          <t>projects/04-columnar-query-engine/backend/tests/sql_tests.rs</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="7" t="inlineStr">
@@ -20603,22 +20859,26 @@
           <t>P0</t>
         </is>
       </c>
-      <c r="D22" s="8" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="E22" s="8" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="D22" s="9" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="E22" s="9" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="F22" s="7" t="inlineStr">
         <is>
-          <t>Specified</t>
-        </is>
-      </c>
-      <c r="G22" s="7" t="inlineStr"/>
+          <t>Verified</t>
+        </is>
+      </c>
+      <c r="G22" s="7" t="inlineStr">
+        <is>
+          <t>projects/04-columnar-query-engine/backend/tests/sql_tests.rs</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="7" t="inlineStr">
@@ -20636,22 +20896,26 @@
           <t>P0</t>
         </is>
       </c>
-      <c r="D23" s="8" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="E23" s="8" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="D23" s="9" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="E23" s="9" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="F23" s="7" t="inlineStr">
         <is>
-          <t>Specified</t>
-        </is>
-      </c>
-      <c r="G23" s="7" t="inlineStr"/>
+          <t>Verified</t>
+        </is>
+      </c>
+      <c r="G23" s="7" t="inlineStr">
+        <is>
+          <t>projects/04-columnar-query-engine/backend/tests/sql_tests.rs</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="7" t="inlineStr">
@@ -20669,22 +20933,26 @@
           <t>P0</t>
         </is>
       </c>
-      <c r="D24" s="8" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="E24" s="8" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="D24" s="9" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="E24" s="9" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="F24" s="7" t="inlineStr">
         <is>
-          <t>Specified</t>
-        </is>
-      </c>
-      <c r="G24" s="7" t="inlineStr"/>
+          <t>Verified</t>
+        </is>
+      </c>
+      <c r="G24" s="7" t="inlineStr">
+        <is>
+          <t>projects/04-columnar-query-engine/backend/tests/sql_tests.rs</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="7" t="inlineStr">
@@ -20776,22 +21044,26 @@
           <t>P0</t>
         </is>
       </c>
-      <c r="D27" s="8" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="E27" s="8" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="D27" s="9" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="E27" s="9" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="F27" s="7" t="inlineStr">
         <is>
-          <t>Specified</t>
-        </is>
-      </c>
-      <c r="G27" s="7" t="inlineStr"/>
+          <t>Verified</t>
+        </is>
+      </c>
+      <c r="G27" s="7" t="inlineStr">
+        <is>
+          <t>projects/04-columnar-query-engine/backend/tests/sql_tests.rs</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="7" t="inlineStr">
@@ -20809,22 +21081,26 @@
           <t>P0</t>
         </is>
       </c>
-      <c r="D28" s="8" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="E28" s="8" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="D28" s="9" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="E28" s="9" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="F28" s="7" t="inlineStr">
         <is>
-          <t>Specified</t>
-        </is>
-      </c>
-      <c r="G28" s="7" t="inlineStr"/>
+          <t>Verified</t>
+        </is>
+      </c>
+      <c r="G28" s="7" t="inlineStr">
+        <is>
+          <t>projects/04-columnar-query-engine/backend/tests/sql_tests.rs</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="7" t="inlineStr">
@@ -21229,22 +21505,26 @@
           <t>P0</t>
         </is>
       </c>
-      <c r="D40" s="8" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="E40" s="8" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="D40" s="9" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="E40" s="9" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="F40" s="7" t="inlineStr">
         <is>
-          <t>Specified</t>
-        </is>
-      </c>
-      <c r="G40" s="7" t="inlineStr"/>
+          <t>Verified</t>
+        </is>
+      </c>
+      <c r="G40" s="7" t="inlineStr">
+        <is>
+          <t>projects/04-columnar-query-engine/backend/tests/sql_tests.rs</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="7" t="inlineStr">
@@ -21587,22 +21867,26 @@
           <t>P0</t>
         </is>
       </c>
-      <c r="D50" s="8" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="E50" s="8" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="D50" s="9" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="E50" s="9" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="F50" s="7" t="inlineStr">
         <is>
-          <t>Specified</t>
-        </is>
-      </c>
-      <c r="G50" s="7" t="inlineStr"/>
+          <t>Verified</t>
+        </is>
+      </c>
+      <c r="G50" s="7" t="inlineStr">
+        <is>
+          <t>projects/04-columnar-query-engine/backend/tests/sql_tests.rs</t>
+        </is>
+      </c>
     </row>
     <row r="51">
       <c r="A51" s="7" t="inlineStr">
@@ -21620,22 +21904,26 @@
           <t>P0</t>
         </is>
       </c>
-      <c r="D51" s="8" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="E51" s="8" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="D51" s="9" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="E51" s="9" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="F51" s="7" t="inlineStr">
         <is>
-          <t>Specified</t>
-        </is>
-      </c>
-      <c r="G51" s="7" t="inlineStr"/>
+          <t>Verified</t>
+        </is>
+      </c>
+      <c r="G51" s="7" t="inlineStr">
+        <is>
+          <t>projects/04-columnar-query-engine/backend/tests/sql_tests.rs</t>
+        </is>
+      </c>
     </row>
     <row r="52">
       <c r="A52" s="7" t="inlineStr">
@@ -21653,22 +21941,26 @@
           <t>P0</t>
         </is>
       </c>
-      <c r="D52" s="8" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="E52" s="8" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="D52" s="9" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="E52" s="9" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="F52" s="7" t="inlineStr">
         <is>
-          <t>Specified</t>
-        </is>
-      </c>
-      <c r="G52" s="7" t="inlineStr"/>
+          <t>Verified</t>
+        </is>
+      </c>
+      <c r="G52" s="7" t="inlineStr">
+        <is>
+          <t>projects/04-columnar-query-engine/backend/tests/sql_tests.rs</t>
+        </is>
+      </c>
     </row>
     <row r="53">
       <c r="A53" s="7" t="inlineStr">
@@ -21686,22 +21978,26 @@
           <t>P0</t>
         </is>
       </c>
-      <c r="D53" s="8" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="E53" s="8" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="D53" s="9" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="E53" s="9" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="F53" s="7" t="inlineStr">
         <is>
-          <t>Specified</t>
-        </is>
-      </c>
-      <c r="G53" s="7" t="inlineStr"/>
+          <t>Verified</t>
+        </is>
+      </c>
+      <c r="G53" s="7" t="inlineStr">
+        <is>
+          <t>projects/04-columnar-query-engine/backend/tests/sql_tests.rs</t>
+        </is>
+      </c>
     </row>
     <row r="54">
       <c r="A54" s="7" t="inlineStr">
@@ -21752,22 +22048,26 @@
           <t>P0</t>
         </is>
       </c>
-      <c r="D55" s="8" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="E55" s="8" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="D55" s="9" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="E55" s="9" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="F55" s="7" t="inlineStr">
         <is>
-          <t>Specified</t>
-        </is>
-      </c>
-      <c r="G55" s="7" t="inlineStr"/>
+          <t>Verified</t>
+        </is>
+      </c>
+      <c r="G55" s="7" t="inlineStr">
+        <is>
+          <t>projects/04-columnar-query-engine/backend/tests/sql_tests.rs</t>
+        </is>
+      </c>
     </row>
     <row r="56">
       <c r="A56" s="7" t="inlineStr">

</xml_diff>

<commit_message>
S11 Part 4: Clean clone CI validation, final report generator, and status sync
</commit_message>
<xml_diff>
--- a/evidence/workbooks/04_Columnar_Query_Engine_ULTIMATE_145_Master_STATUS.xlsx
+++ b/evidence/workbooks/04_Columnar_Query_Engine_ULTIMATE_145_Master_STATUS.xlsx
@@ -3012,7 +3012,7 @@
       </c>
       <c r="N47" s="7" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>5</t>
         </is>
       </c>
     </row>
@@ -3696,23 +3696,31 @@
           <t>04-056</t>
         </is>
       </c>
-      <c r="J60" s="8" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="K60" s="8" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="J60" s="9" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="K60" s="9" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="L60" s="7" t="inlineStr">
         <is>
-          <t>Specified</t>
-        </is>
-      </c>
-      <c r="M60" s="7" t="inlineStr"/>
-      <c r="N60" s="7" t="inlineStr"/>
+          <t>Verified</t>
+        </is>
+      </c>
+      <c r="M60" s="7" t="inlineStr">
+        <is>
+          <t>projects/04-columnar-query-engine/backend/tests/sql_tests.rs</t>
+        </is>
+      </c>
+      <c r="N60" s="7" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
     </row>
     <row r="61">
       <c r="A61" s="3" t="n">
@@ -3896,23 +3904,31 @@
           <t>04-060</t>
         </is>
       </c>
-      <c r="J64" s="8" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="K64" s="8" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="J64" s="9" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="K64" s="9" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="L64" s="7" t="inlineStr">
         <is>
-          <t>Specified</t>
-        </is>
-      </c>
-      <c r="M64" s="7" t="inlineStr"/>
-      <c r="N64" s="7" t="inlineStr"/>
+          <t>Verified</t>
+        </is>
+      </c>
+      <c r="M64" s="7" t="inlineStr">
+        <is>
+          <t>projects/04-columnar-query-engine/backend/tests/sql_tests.rs</t>
+        </is>
+      </c>
+      <c r="N64" s="7" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
     </row>
     <row r="65">
       <c r="A65" s="3" t="n">
@@ -3946,23 +3962,31 @@
           <t>04-061</t>
         </is>
       </c>
-      <c r="J65" s="8" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="K65" s="8" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="J65" s="9" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="K65" s="9" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="L65" s="7" t="inlineStr">
         <is>
-          <t>Specified</t>
-        </is>
-      </c>
-      <c r="M65" s="7" t="inlineStr"/>
-      <c r="N65" s="7" t="inlineStr"/>
+          <t>Verified</t>
+        </is>
+      </c>
+      <c r="M65" s="7" t="inlineStr">
+        <is>
+          <t>projects/04-columnar-query-engine/backend/tests/sql_tests.rs</t>
+        </is>
+      </c>
+      <c r="N65" s="7" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
     </row>
     <row r="66">
       <c r="A66" s="3" t="n">
@@ -3996,23 +4020,31 @@
           <t>04-062</t>
         </is>
       </c>
-      <c r="J66" s="8" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="K66" s="8" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="J66" s="9" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="K66" s="9" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="L66" s="7" t="inlineStr">
         <is>
-          <t>Specified</t>
-        </is>
-      </c>
-      <c r="M66" s="7" t="inlineStr"/>
-      <c r="N66" s="7" t="inlineStr"/>
+          <t>Verified</t>
+        </is>
+      </c>
+      <c r="M66" s="7" t="inlineStr">
+        <is>
+          <t>projects/04-columnar-query-engine/backend/tests/sql_tests.rs</t>
+        </is>
+      </c>
+      <c r="N66" s="7" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
     </row>
     <row r="67">
       <c r="A67" s="3" t="n">
@@ -4704,23 +4736,31 @@
           <t>04-076</t>
         </is>
       </c>
-      <c r="J80" s="8" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="K80" s="8" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="J80" s="9" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="K80" s="9" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="L80" s="7" t="inlineStr">
         <is>
-          <t>Specified</t>
-        </is>
-      </c>
-      <c r="M80" s="7" t="inlineStr"/>
-      <c r="N80" s="7" t="inlineStr"/>
+          <t>Verified</t>
+        </is>
+      </c>
+      <c r="M80" s="7" t="inlineStr">
+        <is>
+          <t>projects/04-columnar-query-engine/backend/tests/sql_tests.rs</t>
+        </is>
+      </c>
+      <c r="N80" s="7" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
     </row>
     <row r="81">
       <c r="A81" s="3" t="n">
@@ -11894,7 +11934,7 @@
       </c>
       <c r="S44" s="7" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>5</t>
         </is>
       </c>
     </row>
@@ -12877,23 +12917,31 @@
           <t>04-056</t>
         </is>
       </c>
-      <c r="O57" s="8" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="P57" s="8" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="O57" s="9" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="P57" s="9" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="Q57" s="7" t="inlineStr">
         <is>
-          <t>Specified</t>
-        </is>
-      </c>
-      <c r="R57" s="7" t="inlineStr"/>
-      <c r="S57" s="7" t="inlineStr"/>
+          <t>Verified</t>
+        </is>
+      </c>
+      <c r="R57" s="7" t="inlineStr">
+        <is>
+          <t>projects/04-columnar-query-engine/backend/tests/sql_tests.rs</t>
+        </is>
+      </c>
+      <c r="S57" s="7" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
     </row>
     <row r="58">
       <c r="A58" s="5" t="n">
@@ -13169,23 +13217,31 @@
           <t>04-060</t>
         </is>
       </c>
-      <c r="O61" s="8" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="P61" s="8" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="O61" s="9" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="P61" s="9" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="Q61" s="7" t="inlineStr">
         <is>
-          <t>Specified</t>
-        </is>
-      </c>
-      <c r="R61" s="7" t="inlineStr"/>
-      <c r="S61" s="7" t="inlineStr"/>
+          <t>Verified</t>
+        </is>
+      </c>
+      <c r="R61" s="7" t="inlineStr">
+        <is>
+          <t>projects/04-columnar-query-engine/backend/tests/sql_tests.rs</t>
+        </is>
+      </c>
+      <c r="S61" s="7" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
     </row>
     <row r="62">
       <c r="A62" s="5" t="n">
@@ -13242,23 +13298,31 @@
           <t>04-061</t>
         </is>
       </c>
-      <c r="O62" s="8" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="P62" s="8" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="O62" s="9" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="P62" s="9" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="Q62" s="7" t="inlineStr">
         <is>
-          <t>Specified</t>
-        </is>
-      </c>
-      <c r="R62" s="7" t="inlineStr"/>
-      <c r="S62" s="7" t="inlineStr"/>
+          <t>Verified</t>
+        </is>
+      </c>
+      <c r="R62" s="7" t="inlineStr">
+        <is>
+          <t>projects/04-columnar-query-engine/backend/tests/sql_tests.rs</t>
+        </is>
+      </c>
+      <c r="S62" s="7" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
     </row>
     <row r="63">
       <c r="A63" s="5" t="n">
@@ -13315,23 +13379,31 @@
           <t>04-062</t>
         </is>
       </c>
-      <c r="O63" s="8" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="P63" s="8" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="O63" s="9" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="P63" s="9" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="Q63" s="7" t="inlineStr">
         <is>
-          <t>Specified</t>
-        </is>
-      </c>
-      <c r="R63" s="7" t="inlineStr"/>
-      <c r="S63" s="7" t="inlineStr"/>
+          <t>Verified</t>
+        </is>
+      </c>
+      <c r="R63" s="7" t="inlineStr">
+        <is>
+          <t>projects/04-columnar-query-engine/backend/tests/sql_tests.rs</t>
+        </is>
+      </c>
+      <c r="S63" s="7" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
     </row>
     <row r="64">
       <c r="A64" s="5" t="n">
@@ -14345,23 +14417,31 @@
           <t>04-076</t>
         </is>
       </c>
-      <c r="O77" s="8" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="P77" s="8" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="O77" s="9" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="P77" s="9" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="Q77" s="7" t="inlineStr">
         <is>
-          <t>Specified</t>
-        </is>
-      </c>
-      <c r="R77" s="7" t="inlineStr"/>
-      <c r="S77" s="7" t="inlineStr"/>
+          <t>Verified</t>
+        </is>
+      </c>
+      <c r="R77" s="7" t="inlineStr">
+        <is>
+          <t>projects/04-columnar-query-engine/backend/tests/sql_tests.rs</t>
+        </is>
+      </c>
+      <c r="S77" s="7" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
     </row>
     <row r="78">
       <c r="A78" s="5" t="n">
@@ -20351,7 +20431,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-10-02 10:47:50</t>
+          <t>2026-10-02 11:47:39</t>
         </is>
       </c>
     </row>
@@ -20363,7 +20443,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>c955892</t>
+          <t>14aeca4</t>
         </is>
       </c>
     </row>
@@ -21373,22 +21453,26 @@
           <t>P0</t>
         </is>
       </c>
-      <c r="D36" s="8" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="E36" s="8" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="D36" s="9" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="E36" s="9" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="F36" s="7" t="inlineStr">
         <is>
-          <t>Specified</t>
-        </is>
-      </c>
-      <c r="G36" s="7" t="inlineStr"/>
+          <t>Verified</t>
+        </is>
+      </c>
+      <c r="G36" s="7" t="inlineStr">
+        <is>
+          <t>projects/04-columnar-query-engine/backend/tests/sql_tests.rs</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="7" t="inlineStr">
@@ -21406,22 +21490,26 @@
           <t>P0</t>
         </is>
       </c>
-      <c r="D37" s="8" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="E37" s="8" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="D37" s="9" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="E37" s="9" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="F37" s="7" t="inlineStr">
         <is>
-          <t>Specified</t>
-        </is>
-      </c>
-      <c r="G37" s="7" t="inlineStr"/>
+          <t>Verified</t>
+        </is>
+      </c>
+      <c r="G37" s="7" t="inlineStr">
+        <is>
+          <t>projects/04-columnar-query-engine/backend/tests/sql_tests.rs</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="7" t="inlineStr">
@@ -21439,22 +21527,26 @@
           <t>P0</t>
         </is>
       </c>
-      <c r="D38" s="8" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="E38" s="8" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="D38" s="9" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="E38" s="9" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="F38" s="7" t="inlineStr">
         <is>
-          <t>Specified</t>
-        </is>
-      </c>
-      <c r="G38" s="7" t="inlineStr"/>
+          <t>Verified</t>
+        </is>
+      </c>
+      <c r="G38" s="7" t="inlineStr">
+        <is>
+          <t>projects/04-columnar-query-engine/backend/tests/sql_tests.rs</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="7" t="inlineStr">
@@ -21472,22 +21564,26 @@
           <t>P0</t>
         </is>
       </c>
-      <c r="D39" s="8" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="E39" s="8" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="D39" s="9" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="E39" s="9" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="F39" s="7" t="inlineStr">
         <is>
-          <t>Specified</t>
-        </is>
-      </c>
-      <c r="G39" s="7" t="inlineStr"/>
+          <t>Verified</t>
+        </is>
+      </c>
+      <c r="G39" s="7" t="inlineStr">
+        <is>
+          <t>projects/04-columnar-query-engine/backend/tests/sql_tests.rs</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="7" t="inlineStr">
@@ -21542,22 +21638,26 @@
           <t>P0</t>
         </is>
       </c>
-      <c r="D41" s="8" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="E41" s="8" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="D41" s="9" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="E41" s="9" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="F41" s="7" t="inlineStr">
         <is>
-          <t>Specified</t>
-        </is>
-      </c>
-      <c r="G41" s="7" t="inlineStr"/>
+          <t>Verified</t>
+        </is>
+      </c>
+      <c r="G41" s="7" t="inlineStr">
+        <is>
+          <t>projects/04-columnar-query-engine/backend/tests/sql_tests.rs</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="7" t="inlineStr">

</xml_diff>

<commit_message>
S11 Part 4: Final evidence, status workbooks, and CI sync
</commit_message>
<xml_diff>
--- a/evidence/workbooks/04_Columnar_Query_Engine_ULTIMATE_145_Master_STATUS.xlsx
+++ b/evidence/workbooks/04_Columnar_Query_Engine_ULTIMATE_145_Master_STATUS.xlsx
@@ -20431,7 +20431,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-10-02 11:47:39</t>
+          <t>2026-10-02 12:00:31</t>
         </is>
       </c>
     </row>
@@ -20443,7 +20443,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>14aeca4</t>
+          <t>5168869</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
SESSION 13: Final build gate, S12b evidence purge, Backend P1 batch (46 features), grounded docs, and handoff
</commit_message>
<xml_diff>
--- a/evidence/workbooks/04_Columnar_Query_Engine_ULTIMATE_145_Master_STATUS.xlsx
+++ b/evidence/workbooks/04_Columnar_Query_Engine_ULTIMATE_145_Master_STATUS.xlsx
@@ -2052,23 +2052,31 @@
           <t>04-026</t>
         </is>
       </c>
-      <c r="J30" s="8" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="K30" s="8" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="J30" s="9" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="K30" s="9" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="L30" s="7" t="inlineStr">
         <is>
-          <t>Specified</t>
-        </is>
-      </c>
-      <c r="M30" s="7" t="inlineStr"/>
-      <c r="N30" s="7" t="inlineStr"/>
+          <t>Verified</t>
+        </is>
+      </c>
+      <c r="M30" s="7" t="inlineStr">
+        <is>
+          <t>projects/04-columnar-query-engine/backend/tests/query_storage_p1_tests.rs</t>
+        </is>
+      </c>
+      <c r="N30" s="7" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="3" t="n">
@@ -2268,23 +2276,31 @@
           <t>04-030</t>
         </is>
       </c>
-      <c r="J34" s="8" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="K34" s="8" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="J34" s="9" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="K34" s="9" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="L34" s="7" t="inlineStr">
         <is>
-          <t>Specified</t>
-        </is>
-      </c>
-      <c r="M34" s="7" t="inlineStr"/>
-      <c r="N34" s="7" t="inlineStr"/>
+          <t>Verified</t>
+        </is>
+      </c>
+      <c r="M34" s="7" t="inlineStr">
+        <is>
+          <t>projects/04-columnar-query-engine/backend/tests/query_storage_p1_tests.rs</t>
+        </is>
+      </c>
+      <c r="N34" s="7" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="3" t="n">
@@ -2318,23 +2334,31 @@
           <t>04-031</t>
         </is>
       </c>
-      <c r="J35" s="8" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="K35" s="8" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="J35" s="9" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="K35" s="9" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="L35" s="7" t="inlineStr">
         <is>
-          <t>Specified</t>
-        </is>
-      </c>
-      <c r="M35" s="7" t="inlineStr"/>
-      <c r="N35" s="7" t="inlineStr"/>
+          <t>Verified</t>
+        </is>
+      </c>
+      <c r="M35" s="7" t="inlineStr">
+        <is>
+          <t>projects/04-columnar-query-engine/backend/tests/query_storage_p1_tests.rs</t>
+        </is>
+      </c>
+      <c r="N35" s="7" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="3" t="n">
@@ -2600,23 +2624,31 @@
           <t>04-036</t>
         </is>
       </c>
-      <c r="J40" s="8" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="K40" s="8" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="J40" s="9" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="K40" s="9" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="L40" s="7" t="inlineStr">
         <is>
-          <t>Specified</t>
-        </is>
-      </c>
-      <c r="M40" s="7" t="inlineStr"/>
-      <c r="N40" s="7" t="inlineStr"/>
+          <t>Verified</t>
+        </is>
+      </c>
+      <c r="M40" s="7" t="inlineStr">
+        <is>
+          <t>projects/04-columnar-query-engine/backend/tests/query_storage_p1_tests.rs</t>
+        </is>
+      </c>
+      <c r="N40" s="7" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="3" t="n">
@@ -3438,23 +3470,31 @@
           <t>04-051</t>
         </is>
       </c>
-      <c r="J55" s="8" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="K55" s="8" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="J55" s="9" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="K55" s="9" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="L55" s="7" t="inlineStr">
         <is>
-          <t>Specified</t>
-        </is>
-      </c>
-      <c r="M55" s="7" t="inlineStr"/>
-      <c r="N55" s="7" t="inlineStr"/>
+          <t>Verified</t>
+        </is>
+      </c>
+      <c r="M55" s="7" t="inlineStr">
+        <is>
+          <t>projects/04-columnar-query-engine/backend/tests/query_storage_p1_tests.rs</t>
+        </is>
+      </c>
+      <c r="N55" s="7" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
     </row>
     <row r="56">
       <c r="A56" s="3" t="n">
@@ -3488,23 +3528,31 @@
           <t>04-052</t>
         </is>
       </c>
-      <c r="J56" s="8" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="K56" s="8" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="J56" s="9" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="K56" s="9" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="L56" s="7" t="inlineStr">
         <is>
-          <t>Specified</t>
-        </is>
-      </c>
-      <c r="M56" s="7" t="inlineStr"/>
-      <c r="N56" s="7" t="inlineStr"/>
+          <t>Verified</t>
+        </is>
+      </c>
+      <c r="M56" s="7" t="inlineStr">
+        <is>
+          <t>projects/04-columnar-query-engine/backend/tests/query_storage_p1_tests.rs</t>
+        </is>
+      </c>
+      <c r="N56" s="7" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
     </row>
     <row r="57">
       <c r="A57" s="3" t="n">
@@ -3588,23 +3636,31 @@
           <t>04-054</t>
         </is>
       </c>
-      <c r="J58" s="8" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="K58" s="8" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="J58" s="9" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="K58" s="9" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="L58" s="7" t="inlineStr">
         <is>
-          <t>Specified</t>
-        </is>
-      </c>
-      <c r="M58" s="7" t="inlineStr"/>
-      <c r="N58" s="7" t="inlineStr"/>
+          <t>Verified</t>
+        </is>
+      </c>
+      <c r="M58" s="7" t="inlineStr">
+        <is>
+          <t>projects/04-columnar-query-engine/backend/tests/query_storage_p1_tests.rs</t>
+        </is>
+      </c>
+      <c r="N58" s="7" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
     </row>
     <row r="59">
       <c r="A59" s="3" t="n">
@@ -3804,23 +3860,31 @@
           <t>04-058</t>
         </is>
       </c>
-      <c r="J62" s="8" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="K62" s="8" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="J62" s="9" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="K62" s="9" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="L62" s="7" t="inlineStr">
         <is>
-          <t>Specified</t>
-        </is>
-      </c>
-      <c r="M62" s="7" t="inlineStr"/>
-      <c r="N62" s="7" t="inlineStr"/>
+          <t>Verified</t>
+        </is>
+      </c>
+      <c r="M62" s="7" t="inlineStr">
+        <is>
+          <t>projects/04-columnar-query-engine/backend/tests/query_storage_p1_tests.rs</t>
+        </is>
+      </c>
+      <c r="N62" s="7" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
     </row>
     <row r="63">
       <c r="A63" s="3" t="n">
@@ -4078,23 +4142,31 @@
           <t>04-063</t>
         </is>
       </c>
-      <c r="J67" s="8" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="K67" s="8" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="J67" s="9" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="K67" s="9" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="L67" s="7" t="inlineStr">
         <is>
-          <t>Specified</t>
-        </is>
-      </c>
-      <c r="M67" s="7" t="inlineStr"/>
-      <c r="N67" s="7" t="inlineStr"/>
+          <t>Verified</t>
+        </is>
+      </c>
+      <c r="M67" s="7" t="inlineStr">
+        <is>
+          <t>projects/04-columnar-query-engine/backend/tests/query_storage_p1_tests.rs</t>
+        </is>
+      </c>
+      <c r="N67" s="7" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
     </row>
     <row r="68">
       <c r="A68" s="3" t="n">
@@ -4128,23 +4200,31 @@
           <t>04-064</t>
         </is>
       </c>
-      <c r="J68" s="8" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="K68" s="8" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="J68" s="9" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="K68" s="9" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="L68" s="7" t="inlineStr">
         <is>
-          <t>Specified</t>
-        </is>
-      </c>
-      <c r="M68" s="7" t="inlineStr"/>
-      <c r="N68" s="7" t="inlineStr"/>
+          <t>Verified</t>
+        </is>
+      </c>
+      <c r="M68" s="7" t="inlineStr">
+        <is>
+          <t>projects/04-columnar-query-engine/backend/tests/query_storage_p1_tests.rs</t>
+        </is>
+      </c>
+      <c r="N68" s="7" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
     </row>
     <row r="69">
       <c r="A69" s="3" t="n">
@@ -4178,23 +4258,31 @@
           <t>04-065</t>
         </is>
       </c>
-      <c r="J69" s="8" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="K69" s="8" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="J69" s="9" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="K69" s="9" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="L69" s="7" t="inlineStr">
         <is>
-          <t>Specified</t>
-        </is>
-      </c>
-      <c r="M69" s="7" t="inlineStr"/>
-      <c r="N69" s="7" t="inlineStr"/>
+          <t>Verified</t>
+        </is>
+      </c>
+      <c r="M69" s="7" t="inlineStr">
+        <is>
+          <t>projects/04-columnar-query-engine/backend/tests/query_storage_p1_tests.rs</t>
+        </is>
+      </c>
+      <c r="N69" s="7" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
     </row>
     <row r="70">
       <c r="A70" s="3" t="n">
@@ -4386,23 +4474,31 @@
           <t>04-069</t>
         </is>
       </c>
-      <c r="J73" s="8" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="K73" s="8" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="J73" s="9" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="K73" s="9" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="L73" s="7" t="inlineStr">
         <is>
-          <t>Specified</t>
-        </is>
-      </c>
-      <c r="M73" s="7" t="inlineStr"/>
-      <c r="N73" s="7" t="inlineStr"/>
+          <t>Verified</t>
+        </is>
+      </c>
+      <c r="M73" s="7" t="inlineStr">
+        <is>
+          <t>projects/04-columnar-query-engine/backend/tests/query_storage_p1_tests.rs</t>
+        </is>
+      </c>
+      <c r="N73" s="7" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
     </row>
     <row r="74">
       <c r="A74" s="3" t="n">
@@ -4436,23 +4532,31 @@
           <t>04-070</t>
         </is>
       </c>
-      <c r="J74" s="8" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="K74" s="8" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="J74" s="9" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="K74" s="9" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="L74" s="7" t="inlineStr">
         <is>
-          <t>Specified</t>
-        </is>
-      </c>
-      <c r="M74" s="7" t="inlineStr"/>
-      <c r="N74" s="7" t="inlineStr"/>
+          <t>Verified</t>
+        </is>
+      </c>
+      <c r="M74" s="7" t="inlineStr">
+        <is>
+          <t>projects/04-columnar-query-engine/backend/tests/query_storage_p1_tests.rs</t>
+        </is>
+      </c>
+      <c r="N74" s="7" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
     </row>
     <row r="75">
       <c r="A75" s="3" t="n">
@@ -5600,23 +5704,31 @@
           <t>04-092</t>
         </is>
       </c>
-      <c r="J96" s="8" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="K96" s="8" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="J96" s="9" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="K96" s="9" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="L96" s="7" t="inlineStr">
         <is>
-          <t>Specified</t>
-        </is>
-      </c>
-      <c r="M96" s="7" t="inlineStr"/>
-      <c r="N96" s="7" t="inlineStr"/>
+          <t>Verified</t>
+        </is>
+      </c>
+      <c r="M96" s="7" t="inlineStr">
+        <is>
+          <t>projects/04-columnar-query-engine/backend/tests/query_storage_p1_tests.rs</t>
+        </is>
+      </c>
+      <c r="N96" s="7" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
     </row>
     <row r="97">
       <c r="A97" s="3" t="n">
@@ -7926,23 +8038,31 @@
           <t>04-135</t>
         </is>
       </c>
-      <c r="J139" s="8" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="K139" s="8" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="J139" s="9" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="K139" s="9" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="L139" s="7" t="inlineStr">
         <is>
-          <t>Specified</t>
-        </is>
-      </c>
-      <c r="M139" s="7" t="inlineStr"/>
-      <c r="N139" s="7" t="inlineStr"/>
+          <t>Verified</t>
+        </is>
+      </c>
+      <c r="M139" s="7" t="inlineStr">
+        <is>
+          <t>projects/04-columnar-query-engine/backend/tests/sql_tests.rs</t>
+        </is>
+      </c>
+      <c r="N139" s="7" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
     </row>
     <row r="140">
       <c r="A140" s="3" t="n">
@@ -10583,23 +10703,31 @@
           <t>04-026</t>
         </is>
       </c>
-      <c r="O27" s="8" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="P27" s="8" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="O27" s="9" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="P27" s="9" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="Q27" s="7" t="inlineStr">
         <is>
-          <t>Specified</t>
-        </is>
-      </c>
-      <c r="R27" s="7" t="inlineStr"/>
-      <c r="S27" s="7" t="inlineStr"/>
+          <t>Verified</t>
+        </is>
+      </c>
+      <c r="R27" s="7" t="inlineStr">
+        <is>
+          <t>projects/04-columnar-query-engine/backend/tests/query_storage_p1_tests.rs</t>
+        </is>
+      </c>
+      <c r="S27" s="7" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="5" t="n">
@@ -10891,23 +11019,31 @@
           <t>04-030</t>
         </is>
       </c>
-      <c r="O31" s="8" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="P31" s="8" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="O31" s="9" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="P31" s="9" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="Q31" s="7" t="inlineStr">
         <is>
-          <t>Specified</t>
-        </is>
-      </c>
-      <c r="R31" s="7" t="inlineStr"/>
-      <c r="S31" s="7" t="inlineStr"/>
+          <t>Verified</t>
+        </is>
+      </c>
+      <c r="R31" s="7" t="inlineStr">
+        <is>
+          <t>projects/04-columnar-query-engine/backend/tests/query_storage_p1_tests.rs</t>
+        </is>
+      </c>
+      <c r="S31" s="7" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="5" t="n">
@@ -10964,23 +11100,31 @@
           <t>04-031</t>
         </is>
       </c>
-      <c r="O32" s="8" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="P32" s="8" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="O32" s="9" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="P32" s="9" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="Q32" s="7" t="inlineStr">
         <is>
-          <t>Specified</t>
-        </is>
-      </c>
-      <c r="R32" s="7" t="inlineStr"/>
-      <c r="S32" s="7" t="inlineStr"/>
+          <t>Verified</t>
+        </is>
+      </c>
+      <c r="R32" s="7" t="inlineStr">
+        <is>
+          <t>projects/04-columnar-query-engine/backend/tests/query_storage_p1_tests.rs</t>
+        </is>
+      </c>
+      <c r="S32" s="7" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="5" t="n">
@@ -11361,23 +11505,31 @@
           <t>04-036</t>
         </is>
       </c>
-      <c r="O37" s="8" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="P37" s="8" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="O37" s="9" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="P37" s="9" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="Q37" s="7" t="inlineStr">
         <is>
-          <t>Specified</t>
-        </is>
-      </c>
-      <c r="R37" s="7" t="inlineStr"/>
-      <c r="S37" s="7" t="inlineStr"/>
+          <t>Verified</t>
+        </is>
+      </c>
+      <c r="R37" s="7" t="inlineStr">
+        <is>
+          <t>projects/04-columnar-query-engine/backend/tests/query_storage_p1_tests.rs</t>
+        </is>
+      </c>
+      <c r="S37" s="7" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="5" t="n">
@@ -12544,23 +12696,31 @@
           <t>04-051</t>
         </is>
       </c>
-      <c r="O52" s="8" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="P52" s="8" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="O52" s="9" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="P52" s="9" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="Q52" s="7" t="inlineStr">
         <is>
-          <t>Specified</t>
-        </is>
-      </c>
-      <c r="R52" s="7" t="inlineStr"/>
-      <c r="S52" s="7" t="inlineStr"/>
+          <t>Verified</t>
+        </is>
+      </c>
+      <c r="R52" s="7" t="inlineStr">
+        <is>
+          <t>projects/04-columnar-query-engine/backend/tests/query_storage_p1_tests.rs</t>
+        </is>
+      </c>
+      <c r="S52" s="7" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
     </row>
     <row r="53">
       <c r="A53" s="5" t="n">
@@ -12617,23 +12777,31 @@
           <t>04-052</t>
         </is>
       </c>
-      <c r="O53" s="8" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="P53" s="8" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="O53" s="9" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="P53" s="9" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="Q53" s="7" t="inlineStr">
         <is>
-          <t>Specified</t>
-        </is>
-      </c>
-      <c r="R53" s="7" t="inlineStr"/>
-      <c r="S53" s="7" t="inlineStr"/>
+          <t>Verified</t>
+        </is>
+      </c>
+      <c r="R53" s="7" t="inlineStr">
+        <is>
+          <t>projects/04-columnar-query-engine/backend/tests/query_storage_p1_tests.rs</t>
+        </is>
+      </c>
+      <c r="S53" s="7" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
     </row>
     <row r="54">
       <c r="A54" s="5" t="n">
@@ -12763,23 +12931,31 @@
           <t>04-054</t>
         </is>
       </c>
-      <c r="O55" s="8" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="P55" s="8" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="O55" s="9" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="P55" s="9" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="Q55" s="7" t="inlineStr">
         <is>
-          <t>Specified</t>
-        </is>
-      </c>
-      <c r="R55" s="7" t="inlineStr"/>
-      <c r="S55" s="7" t="inlineStr"/>
+          <t>Verified</t>
+        </is>
+      </c>
+      <c r="R55" s="7" t="inlineStr">
+        <is>
+          <t>projects/04-columnar-query-engine/backend/tests/query_storage_p1_tests.rs</t>
+        </is>
+      </c>
+      <c r="S55" s="7" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
     </row>
     <row r="56">
       <c r="A56" s="5" t="n">
@@ -13071,23 +13247,31 @@
           <t>04-058</t>
         </is>
       </c>
-      <c r="O59" s="8" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="P59" s="8" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="O59" s="9" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="P59" s="9" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="Q59" s="7" t="inlineStr">
         <is>
-          <t>Specified</t>
-        </is>
-      </c>
-      <c r="R59" s="7" t="inlineStr"/>
-      <c r="S59" s="7" t="inlineStr"/>
+          <t>Verified</t>
+        </is>
+      </c>
+      <c r="R59" s="7" t="inlineStr">
+        <is>
+          <t>projects/04-columnar-query-engine/backend/tests/query_storage_p1_tests.rs</t>
+        </is>
+      </c>
+      <c r="S59" s="7" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
     </row>
     <row r="60">
       <c r="A60" s="5" t="n">
@@ -13460,23 +13644,31 @@
           <t>04-063</t>
         </is>
       </c>
-      <c r="O64" s="8" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="P64" s="8" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="O64" s="9" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="P64" s="9" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="Q64" s="7" t="inlineStr">
         <is>
-          <t>Specified</t>
-        </is>
-      </c>
-      <c r="R64" s="7" t="inlineStr"/>
-      <c r="S64" s="7" t="inlineStr"/>
+          <t>Verified</t>
+        </is>
+      </c>
+      <c r="R64" s="7" t="inlineStr">
+        <is>
+          <t>projects/04-columnar-query-engine/backend/tests/query_storage_p1_tests.rs</t>
+        </is>
+      </c>
+      <c r="S64" s="7" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
     </row>
     <row r="65">
       <c r="A65" s="5" t="n">
@@ -13533,23 +13725,31 @@
           <t>04-064</t>
         </is>
       </c>
-      <c r="O65" s="8" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="P65" s="8" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="O65" s="9" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="P65" s="9" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="Q65" s="7" t="inlineStr">
         <is>
-          <t>Specified</t>
-        </is>
-      </c>
-      <c r="R65" s="7" t="inlineStr"/>
-      <c r="S65" s="7" t="inlineStr"/>
+          <t>Verified</t>
+        </is>
+      </c>
+      <c r="R65" s="7" t="inlineStr">
+        <is>
+          <t>projects/04-columnar-query-engine/backend/tests/query_storage_p1_tests.rs</t>
+        </is>
+      </c>
+      <c r="S65" s="7" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
     </row>
     <row r="66">
       <c r="A66" s="5" t="n">
@@ -13606,23 +13806,31 @@
           <t>04-065</t>
         </is>
       </c>
-      <c r="O66" s="8" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="P66" s="8" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="O66" s="9" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="P66" s="9" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="Q66" s="7" t="inlineStr">
         <is>
-          <t>Specified</t>
-        </is>
-      </c>
-      <c r="R66" s="7" t="inlineStr"/>
-      <c r="S66" s="7" t="inlineStr"/>
+          <t>Verified</t>
+        </is>
+      </c>
+      <c r="R66" s="7" t="inlineStr">
+        <is>
+          <t>projects/04-columnar-query-engine/backend/tests/query_storage_p1_tests.rs</t>
+        </is>
+      </c>
+      <c r="S66" s="7" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
     </row>
     <row r="67">
       <c r="A67" s="5" t="n">
@@ -13906,23 +14114,31 @@
           <t>04-069</t>
         </is>
       </c>
-      <c r="O70" s="8" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="P70" s="8" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="O70" s="9" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="P70" s="9" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="Q70" s="7" t="inlineStr">
         <is>
-          <t>Specified</t>
-        </is>
-      </c>
-      <c r="R70" s="7" t="inlineStr"/>
-      <c r="S70" s="7" t="inlineStr"/>
+          <t>Verified</t>
+        </is>
+      </c>
+      <c r="R70" s="7" t="inlineStr">
+        <is>
+          <t>projects/04-columnar-query-engine/backend/tests/query_storage_p1_tests.rs</t>
+        </is>
+      </c>
+      <c r="S70" s="7" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
     </row>
     <row r="71">
       <c r="A71" s="5" t="n">
@@ -13979,23 +14195,31 @@
           <t>04-070</t>
         </is>
       </c>
-      <c r="O71" s="8" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="P71" s="8" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="O71" s="9" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="P71" s="9" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="Q71" s="7" t="inlineStr">
         <is>
-          <t>Specified</t>
-        </is>
-      </c>
-      <c r="R71" s="7" t="inlineStr"/>
-      <c r="S71" s="7" t="inlineStr"/>
+          <t>Verified</t>
+        </is>
+      </c>
+      <c r="R71" s="7" t="inlineStr">
+        <is>
+          <t>projects/04-columnar-query-engine/backend/tests/query_storage_p1_tests.rs</t>
+        </is>
+      </c>
+      <c r="S71" s="7" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
     </row>
     <row r="72">
       <c r="A72" s="5" t="n">
@@ -15649,23 +15873,31 @@
           <t>04-092</t>
         </is>
       </c>
-      <c r="O93" s="8" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="P93" s="8" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="O93" s="9" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="P93" s="9" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="Q93" s="7" t="inlineStr">
         <is>
-          <t>Specified</t>
-        </is>
-      </c>
-      <c r="R93" s="7" t="inlineStr"/>
-      <c r="S93" s="7" t="inlineStr"/>
+          <t>Verified</t>
+        </is>
+      </c>
+      <c r="R93" s="7" t="inlineStr">
+        <is>
+          <t>projects/04-columnar-query-engine/backend/tests/query_storage_p1_tests.rs</t>
+        </is>
+      </c>
+      <c r="S93" s="7" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
     </row>
     <row r="94">
       <c r="A94" s="5" t="n">
@@ -18964,23 +19196,31 @@
           <t>04-135</t>
         </is>
       </c>
-      <c r="O136" s="8" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="P136" s="8" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="O136" s="9" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="P136" s="9" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="Q136" s="7" t="inlineStr">
         <is>
-          <t>Specified</t>
-        </is>
-      </c>
-      <c r="R136" s="7" t="inlineStr"/>
-      <c r="S136" s="7" t="inlineStr"/>
+          <t>Verified</t>
+        </is>
+      </c>
+      <c r="R136" s="7" t="inlineStr">
+        <is>
+          <t>projects/04-columnar-query-engine/backend/tests/sql_tests.rs</t>
+        </is>
+      </c>
+      <c r="S136" s="7" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
     </row>
     <row r="137">
       <c r="A137" s="5" t="n">
@@ -20431,7 +20671,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-10-02 12:00:31</t>
+          <t>2026-10-02 20:05:03</t>
         </is>
       </c>
     </row>
@@ -20443,7 +20683,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>5168869</t>
+          <t>2700149</t>
         </is>
       </c>
     </row>
@@ -22185,22 +22425,26 @@
           <t>P0</t>
         </is>
       </c>
-      <c r="D56" s="8" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="E56" s="8" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="D56" s="9" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="E56" s="9" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="F56" s="7" t="inlineStr">
         <is>
-          <t>Specified</t>
-        </is>
-      </c>
-      <c r="G56" s="7" t="inlineStr"/>
+          <t>Verified</t>
+        </is>
+      </c>
+      <c r="G56" s="7" t="inlineStr">
+        <is>
+          <t>projects/04-columnar-query-engine/backend/tests/sql_tests.rs</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="1">

</xml_diff>